<commit_message>
Rekenboek v3.1: kolom Betekenis bij de ontwerpresultaten ingevuld
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Onderbouwing/Rekenboek_herontwerp_v3.1.xlsx
+++ b/Onderbouwing/Rekenboek_herontwerp_v3.1.xlsx
@@ -908,7 +908,7 @@
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
     <col width="68" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1033,7 +1033,11 @@
         <f>'Containers'!F15</f>
         <v/>
       </c>
-      <c r="G6" s="9" t="n"/>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Aantal containerligplaatsen dat nodig is om de overslag te halen bij max. 65% kadebezetting.</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="n"/>
     </row>
     <row r="7" ht="27" customHeight="1">
@@ -1064,7 +1068,11 @@
         <f>'Containers'!F16</f>
         <v/>
       </c>
-      <c r="G7" s="9" t="n"/>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Aantal getekende ligplaatsen (C1-C4); gelijk aan of meer dan vereist = voldoet.</t>
+        </is>
+      </c>
       <c r="H7" s="9" t="n"/>
     </row>
     <row r="8" ht="27" customHeight="1">
@@ -1095,7 +1103,11 @@
         <f>'Containers'!F17</f>
         <v/>
       </c>
-      <c r="G8" s="9" t="n"/>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Deel van de tijd dat de kade bezet is; onder 65% blijven de wachttijden voor schepen beperkt.</t>
+        </is>
+      </c>
       <c r="H8" s="9" t="n"/>
     </row>
     <row r="9" ht="27" customHeight="1">
@@ -1126,7 +1138,11 @@
         <f>'Containers'!F18</f>
         <v/>
       </c>
-      <c r="G9" s="9" t="n"/>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Getekende kadelengte (4 x ca. 401 m); ruim voor 4 schepen van 334 m met tussenruimte.</t>
+        </is>
+      </c>
       <c r="H9" s="9" t="n"/>
     </row>
     <row r="10" ht="27" customHeight="1">
@@ -1157,7 +1173,11 @@
         <f>'Containers'!F19</f>
         <v/>
       </c>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Aantal STS-kranen dat tegelijk werkt (3/4/5 per schip); in de eindfase 20 getekend.</t>
+        </is>
+      </c>
       <c r="H10" s="9" t="n"/>
     </row>
     <row r="11" ht="27" customHeight="1">
@@ -1188,7 +1208,11 @@
         <f>'Containers'!F27</f>
         <v/>
       </c>
-      <c r="G11" s="9" t="n"/>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Benodigd containerterrein uit voorraad, stapeling en terreinfactor.</t>
+        </is>
+      </c>
       <c r="H11" s="9" t="n"/>
     </row>
     <row r="12" ht="27" customHeight="1">
@@ -1219,7 +1243,11 @@
         <f>'Containers'!F28</f>
         <v/>
       </c>
-      <c r="G12" s="9" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Getekend containerterrein; groter dan nodig = ruimte voor gate, spoor en buffers.</t>
+        </is>
+      </c>
       <c r="H12" s="9" t="n"/>
     </row>
     <row r="13" ht="27" customHeight="1">
@@ -1250,7 +1278,11 @@
         <f>'Overige terminals'!F10</f>
         <v/>
       </c>
-      <c r="G13" s="9" t="n"/>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Graanterrein volgens het oude rekenmodel (8 m opslaghoogte); getekend is 30,4 ha met silo s en loods.</t>
+        </is>
+      </c>
       <c r="H13" s="9" t="n"/>
     </row>
     <row r="14" ht="27" customHeight="1">
@@ -1281,7 +1313,11 @@
         <f>'Overige terminals'!F16</f>
         <v/>
       </c>
-      <c r="G14" s="9" t="n"/>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Benodigd RoRo-terrein voor de autovoorraad; getekend is 30,2 ha = voldoet.</t>
+        </is>
+      </c>
       <c r="H14" s="9" t="n"/>
     </row>
     <row r="15" ht="27" customHeight="1">
@@ -1312,7 +1348,11 @@
         <f>'Overige terminals'!F19</f>
         <v/>
       </c>
-      <c r="G15" s="9" t="n"/>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Aantal LNG-schepen per jaar (ca. 1 per week in 2045).</t>
+        </is>
+      </c>
       <c r="H15" s="9" t="n"/>
     </row>
     <row r="16" ht="27" customHeight="1">
@@ -1343,7 +1383,11 @@
         <f>'Overige terminals'!F25</f>
         <v/>
       </c>
-      <c r="G16" s="9" t="n"/>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Vrije tankruimte bij aankomst van een volle LNG-tanker; positief = de lading past.</t>
+        </is>
+      </c>
       <c r="H16" s="9" t="n"/>
     </row>
     <row r="17" ht="27" customHeight="1">
@@ -1374,7 +1418,11 @@
         <f>'Overige terminals'!F27</f>
         <v/>
       </c>
-      <c r="G17" s="9" t="n"/>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Idem als één tank buiten bedrijf is (N-1). Negatief in 2045 = de gereserveerde 4e tank is dan nodig.</t>
+        </is>
+      </c>
       <c r="H17" s="9" t="n"/>
     </row>
     <row r="18" ht="27" customHeight="1">
@@ -1405,7 +1453,11 @@
         <f>'Overige terminals'!F30</f>
         <v/>
       </c>
-      <c r="G18" s="9" t="n"/>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Elektrisch vermogen van de gascentrale als 50% van het LNG naar de centrale gaat (rekenvoorbeeld).</t>
+        </is>
+      </c>
       <c r="H18" s="9" t="n"/>
     </row>
     <row r="19" ht="27" customHeight="1">

</xml_diff>